<commit_message>
correct some mistakes in the tested-exploit-list
</commit_message>
<xml_diff>
--- a/1-func-test/Tested-Exploit-List.xlsx
+++ b/1-func-test/Tested-Exploit-List.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\陈铂英\Desktop\kShield\1-func-test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{698A24CD-DDED-4C35-88DC-B9D84C2CDA85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D77ADEE3-09CE-4A4F-8528-0239FE12BDF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_1" localSheetId="0">sheet1!$B$4:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sheet1!$A$3:$M$19</definedName>
+    <definedName name="_1" localSheetId="0">sheet1!$B$6:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sheet1!$A$3:$M$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">sheet1!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="89">
   <si>
     <t>影响</t>
   </si>
@@ -356,6 +356,50 @@
   </si>
   <si>
     <t>The exploit is unstable, but testing has confirmed that it can be successfully exploited. After adding protections, it can also be successfully mitigated.</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>CVE-2020-8835</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>CVE-2021-43267</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>CVE-2020-27194</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Linux-5.8.14</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Integer truncation in the eBPF verifier's `scalar32_min_max_or()` function, caused by assigning a 64-bit value to a 32-bit variable during OR operations, leads to incorrect register range calculation</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Improper conversion of 64-bit values to 32-bit (by directly taking the lower 32 bits) causes inconsistency between the BPF verification and execution phases, leading to out-of-bounds reads/writes.</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Linux-5.5.0</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>An incorrect length validation for MSG_CRYPTO messages in the TIPC (Transparent Inter-Process Communication) intra-cluster protocol results in heap overflow.</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Linux-5.14.15</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>cannot extract BTF info from the provided bzimage, but the principle of this exploit is as the same as CVE-2020-27194, and thus can be detected and eliminated by kshield.</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>the provided bzimage doesn't include symbol for modprobe_path but the principle of this exploit is as the same as other modprobe_path overwrite exploits. Thus it can be detected and eliminated by kshield.</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
@@ -526,7 +570,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -576,9 +620,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -593,6 +634,21 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -998,7 +1054,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.75" style="1" customWidth="1"/>
@@ -1017,53 +1073,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="18"/>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
+      <c r="A1" s="17"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
       <c r="M1" s="9"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="21" t="s">
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="20" t="s">
         <v>43</v>
       </c>
       <c r="I2" s="3"/>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="K2" s="20" t="s">
+      <c r="K2" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
     </row>
     <row r="3" spans="1:13" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="22"/>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
+      <c r="A3" s="21"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
       <c r="D3" s="5">
         <v>4.1900000000000004</v>
       </c>
@@ -1076,11 +1132,11 @@
       <c r="G3" s="5">
         <v>5.12</v>
       </c>
-      <c r="H3" s="22"/>
+      <c r="H3" s="21"/>
       <c r="I3" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="22"/>
+      <c r="J3" s="21"/>
       <c r="K3" s="10" t="s">
         <v>46</v>
       </c>
@@ -1091,33 +1147,23 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="78" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
-        <v>2</v>
+    <row r="4" spans="1:13" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="14" t="s">
+        <v>78</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="7">
-        <v>1</v>
-      </c>
-      <c r="E4" s="7">
-        <v>1</v>
-      </c>
-      <c r="F4" s="7">
-        <v>1</v>
-      </c>
-      <c r="G4" s="7">
-        <v>1</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>4</v>
+        <v>83</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="13" t="s">
+        <v>50</v>
       </c>
       <c r="J4" s="13" t="s">
         <v>52</v>
@@ -1128,56 +1174,47 @@
       <c r="L4" s="7">
         <v>1</v>
       </c>
-      <c r="M4" s="12"/>
-    </row>
-    <row r="5" spans="1:13" ht="79.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="7">
-        <v>1</v>
-      </c>
-      <c r="E5" s="7">
-        <v>1</v>
-      </c>
-      <c r="F5" s="7">
-        <v>1</v>
-      </c>
-      <c r="G5" s="7">
-        <v>1</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>4</v>
+      <c r="M4" s="15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="78" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="I5" s="13" t="s">
+        <v>50</v>
       </c>
       <c r="J5" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="K5" s="7">
-        <v>1</v>
-      </c>
-      <c r="L5" s="7">
-        <v>1</v>
-      </c>
-      <c r="M5" s="12"/>
-    </row>
-    <row r="6" spans="1:13" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="K5" s="24">
+        <v>1</v>
+      </c>
+      <c r="L5" s="24">
+        <v>1</v>
+      </c>
+      <c r="M5" s="23"/>
+    </row>
+    <row r="6" spans="1:13" ht="78" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D6" s="7">
         <v>1</v>
@@ -1191,7 +1228,9 @@
       <c r="G6" s="7">
         <v>1</v>
       </c>
-      <c r="H6" s="6"/>
+      <c r="H6" s="14" t="s">
+        <v>74</v>
+      </c>
       <c r="I6" s="7" t="s">
         <v>4</v>
       </c>
@@ -1206,64 +1245,64 @@
       </c>
       <c r="M6" s="12"/>
     </row>
-    <row r="7" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
-        <v>9</v>
+    <row r="7" spans="1:13" ht="80.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="14" t="s">
+        <v>79</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>10</v>
+        <v>85</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>86</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
-      <c r="H7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" s="11" t="s">
+      <c r="H7" s="14"/>
+      <c r="I7" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" s="7">
+        <v>1</v>
+      </c>
+      <c r="L7" s="7">
+        <v>1</v>
+      </c>
+      <c r="M7" s="15" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="79.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="7">
+        <v>1</v>
+      </c>
+      <c r="E8" s="7">
+        <v>1</v>
+      </c>
+      <c r="F8" s="7">
+        <v>1</v>
+      </c>
+      <c r="G8" s="7">
+        <v>1</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="I8" s="7" t="s">
         <v>4</v>
-      </c>
-      <c r="J7" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="K7" s="7">
-        <v>1</v>
-      </c>
-      <c r="L7" s="7">
-        <v>1</v>
-      </c>
-      <c r="M7" s="7"/>
-    </row>
-    <row r="8" spans="1:13" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="7">
-        <v>0</v>
-      </c>
-      <c r="E8" s="7">
-        <v>0</v>
-      </c>
-      <c r="F8" s="7">
-        <v>1</v>
-      </c>
-      <c r="G8" s="7">
-        <v>1</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="I8" s="13" t="s">
-        <v>50</v>
       </c>
       <c r="J8" s="13" t="s">
         <v>52</v>
@@ -1276,33 +1315,31 @@
       </c>
       <c r="M8" s="12"/>
     </row>
-    <row r="9" spans="1:13" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D9" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="7">
         <v>1</v>
       </c>
       <c r="G9" s="7">
-        <v>0</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>50</v>
+        <v>1</v>
+      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="J9" s="13" t="s">
         <v>52</v>
@@ -1315,62 +1352,64 @@
       </c>
       <c r="M9" s="12"/>
     </row>
-    <row r="10" spans="1:13" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="7">
+        <v>10</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="J10" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="K10" s="7">
+        <v>1</v>
+      </c>
+      <c r="L10" s="7">
+        <v>1</v>
+      </c>
+      <c r="M10" s="7"/>
+    </row>
+    <row r="11" spans="1:13" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="7">
         <v>0</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E11" s="7">
         <v>0</v>
       </c>
-      <c r="F10" s="7">
-        <v>1</v>
-      </c>
-      <c r="G10" s="7">
-        <v>0</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="I10" s="13" t="s">
+      <c r="F11" s="7">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7">
+        <v>1</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" s="13" t="s">
         <v>50</v>
-      </c>
-      <c r="J10" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="K10" s="7">
-        <v>1</v>
-      </c>
-      <c r="L10" s="7">
-        <v>1</v>
-      </c>
-      <c r="M10" s="12"/>
-    </row>
-    <row r="11" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="13" t="s">
-        <v>53</v>
       </c>
       <c r="J11" s="13" t="s">
         <v>52</v>
@@ -1383,33 +1422,33 @@
       </c>
       <c r="M11" s="12"/>
     </row>
-    <row r="12" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D12" s="7">
         <v>0</v>
       </c>
       <c r="E12" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="7">
         <v>1</v>
       </c>
       <c r="G12" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J12" s="13" t="s">
         <v>52</v>
@@ -1422,33 +1461,33 @@
       </c>
       <c r="M12" s="12"/>
     </row>
-    <row r="13" spans="1:13" ht="71.25" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D13" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="7">
         <v>1</v>
       </c>
       <c r="G13" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J13" s="13" t="s">
         <v>52</v>
@@ -1459,32 +1498,22 @@
       <c r="L13" s="7">
         <v>1</v>
       </c>
-      <c r="M13" s="15" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M13" s="12"/>
+    </row>
+    <row r="14" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" s="7">
-        <v>1</v>
-      </c>
-      <c r="E14" s="7">
-        <v>1</v>
-      </c>
-      <c r="F14" s="7">
-        <v>1</v>
-      </c>
-      <c r="G14" s="7">
-        <v>1</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
       <c r="H14" s="6"/>
       <c r="I14" s="13" t="s">
         <v>53</v>
@@ -1500,29 +1529,33 @@
       </c>
       <c r="M14" s="12"/>
     </row>
-    <row r="15" spans="1:13" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6">
-        <v>7.8</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H15" s="6"/>
-      <c r="I15" s="7" t="s">
-        <v>30</v>
+        <v>21</v>
+      </c>
+      <c r="D15" s="7">
+        <v>0</v>
+      </c>
+      <c r="E15" s="7">
+        <v>1</v>
+      </c>
+      <c r="F15" s="7">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7">
+        <v>1</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" s="13" t="s">
+        <v>53</v>
       </c>
       <c r="J15" s="13" t="s">
         <v>52</v>
@@ -1533,31 +1566,35 @@
       <c r="L15" s="7">
         <v>1</v>
       </c>
-      <c r="M15" s="15" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M15" s="12"/>
+    </row>
+    <row r="16" spans="1:13" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="6">
-        <v>5.15</v>
-      </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="7" t="s">
-        <v>30</v>
+        <v>23</v>
+      </c>
+      <c r="D16" s="7">
+        <v>1</v>
+      </c>
+      <c r="E16" s="7">
+        <v>1</v>
+      </c>
+      <c r="F16" s="7">
+        <v>1</v>
+      </c>
+      <c r="G16" s="7">
+        <v>1</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I16" s="13" t="s">
+        <v>53</v>
       </c>
       <c r="J16" s="13" t="s">
         <v>52</v>
@@ -1568,27 +1605,35 @@
       <c r="L16" s="7">
         <v>1</v>
       </c>
-      <c r="M16" s="12"/>
-    </row>
-    <row r="17" spans="1:13" ht="55.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M16" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
+        <v>25</v>
+      </c>
+      <c r="D17" s="7">
+        <v>1</v>
+      </c>
+      <c r="E17" s="7">
+        <v>1</v>
+      </c>
+      <c r="F17" s="7">
+        <v>1</v>
+      </c>
+      <c r="G17" s="7">
+        <v>1</v>
+      </c>
       <c r="H17" s="6"/>
-      <c r="I17" s="7" t="s">
-        <v>30</v>
+      <c r="I17" s="13" t="s">
+        <v>53</v>
       </c>
       <c r="J17" s="13" t="s">
         <v>52</v>
@@ -1599,35 +1644,29 @@
       <c r="L17" s="7">
         <v>1</v>
       </c>
-      <c r="M17" s="15" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M17" s="12"/>
+    </row>
+    <row r="18" spans="1:13" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D18" s="7">
-        <v>0</v>
-      </c>
-      <c r="E18" s="7">
-        <v>1</v>
-      </c>
-      <c r="F18" s="7">
-        <v>1</v>
-      </c>
-      <c r="G18" s="7">
-        <v>1</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>71</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6">
+        <v>7.8</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H18" s="6"/>
       <c r="I18" s="7" t="s">
         <v>30</v>
       </c>
@@ -1644,43 +1683,150 @@
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="136.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="6">
+        <v>5.15</v>
+      </c>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="K19" s="7">
+        <v>1</v>
+      </c>
+      <c r="L19" s="7">
+        <v>1</v>
+      </c>
+      <c r="M19" s="12"/>
+    </row>
+    <row r="20" spans="1:13" ht="55.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="J20" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="K20" s="7">
+        <v>1</v>
+      </c>
+      <c r="L20" s="7">
+        <v>1</v>
+      </c>
+      <c r="M20" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" s="7">
+        <v>0</v>
+      </c>
+      <c r="E21" s="7">
+        <v>1</v>
+      </c>
+      <c r="F21" s="7">
+        <v>1</v>
+      </c>
+      <c r="G21" s="7">
+        <v>1</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="J21" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="K21" s="7">
+        <v>1</v>
+      </c>
+      <c r="L21" s="7">
+        <v>1</v>
+      </c>
+      <c r="M21" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="136.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B22" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="14" t="s">
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="I19" s="13" t="s">
+      <c r="I22" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="J19" s="16" t="s">
+      <c r="J22" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="K19" s="7">
-        <v>1</v>
-      </c>
-      <c r="L19" s="7">
-        <v>1</v>
-      </c>
-      <c r="M19" s="17" t="s">
+      <c r="K22" s="7">
+        <v>1</v>
+      </c>
+      <c r="L22" s="7">
+        <v>1</v>
+      </c>
+      <c r="M22" s="26" t="s">
         <v>75</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M19" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:M19">
-      <sortCondition ref="I3:I46"/>
+  <autoFilter ref="A3:M22" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:M22">
+      <sortCondition ref="I3:I49"/>
     </sortState>
   </autoFilter>
   <mergeCells count="8">
@@ -1694,39 +1840,39 @@
     <mergeCell ref="J2:J3"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
-  <conditionalFormatting sqref="A11:A14">
+  <conditionalFormatting sqref="A14:A17">
     <cfRule type="duplicateValues" dxfId="11" priority="33"/>
     <cfRule type="duplicateValues" dxfId="10" priority="34"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A15:A17">
+  <conditionalFormatting sqref="A18:A20">
     <cfRule type="duplicateValues" dxfId="9" priority="4"/>
     <cfRule type="duplicateValues" dxfId="8" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A18">
+  <conditionalFormatting sqref="A21">
     <cfRule type="duplicateValues" dxfId="7" priority="2"/>
     <cfRule type="duplicateValues" dxfId="6" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A19">
+  <conditionalFormatting sqref="A22">
     <cfRule type="duplicateValues" dxfId="5" priority="29"/>
     <cfRule type="duplicateValues" dxfId="4" priority="30"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A20:A1048576 A1:A10">
+  <conditionalFormatting sqref="A23:A1048576 A1:A13">
     <cfRule type="duplicateValues" dxfId="3" priority="21"/>
     <cfRule type="duplicateValues" dxfId="2" priority="22"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:G14">
+  <conditionalFormatting sqref="D1:G17">
     <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D18:G1048576">
+  <conditionalFormatting sqref="D21:G1048576">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="H7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="J19" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="H10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="J22" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.196850393700787" right="0.196850393700787" top="0.196850393700787" bottom="0.196850393700787" header="0.196850393700787" footer="0.196850393700787"/>

</xml_diff>